<commit_message>
Think3D repro: tables refreshed after re-running blank-render samples
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/think3d_repro/outputs/run1/vlmeval_runs/SPAgent_4B_pi3x_spatial/BLINK/SPAgent_4B_pi3x_spatial_BLINK.xlsx
+++ b/think3d_repro/outputs/run1/vlmeval_runs/SPAgent_4B_pi3x_spatial/BLINK/SPAgent_4B_pi3x_spatial_BLINK.xlsx
@@ -1543,9 +1543,8 @@
 &lt;answer&gt;(A) left&lt;/answer&gt;</t>
   </si>
   <si>
-    <t>The two images show the same bottle of soy sauce (labelled "金标生抽") on a supermarket shelf, with the first image showing the bottle from the left side and the second image showing it from the right side. The camera has moved from a position where the bottle is on the left to a position where it is on the right, indicating a counter-clockwise (left) rotation.
-Therefore, the camera is moving **left**.
-&lt;answer&gt;(A) left&lt;/answer&gt;</t>
+    <t>The 3D reconstruction shows the camera (Cam1*) positioned to the left of the object (bottle), with the object appearing to the right of the camera’s view. The camera’s viewpoint is aligned with the object’s left side, meaning the camera is orbiting the object in a counter-clockwise direction (right turn). The object's label orientation and the background shelf arrangement confirm the camera is moving from the left side of the object to the right side, consistent with a rightward orbit.
+&lt;answer&gt;B&lt;/answer&gt;</t>
   </si>
   <si>
     <t>&lt;think&gt;
@@ -1625,10 +1624,11 @@
 &lt;answer&gt;(B) right&lt;/answer&gt;</t>
   </si>
   <si>
-    <t>The two images show a static scene with a green cup on a table. The first image (left) shows the cup with its handle on the left side of the frame, and the second image (right) shows the cup with its handle on the right side of the frame. This indicates that the camera has moved around the cup in a clockwise direction (left), as the cup appears to rotate in the field of view.
-In the 3D reconstruction, the first image corresponds to the camera position that is looking from the left side of the cup, and the second image corresponds to the camera position that is looking from the right side of the cup. This is consistent with a clockwise rotation (left).
-Therefore, the camera is moving left.
-&lt;answer&gt;A&lt;/answer&gt;</t>
+    <t>The 3D reconstruction shows two camera positions: Cam1 (first image) and Cam2 (second image). The camera orbit is defined by the ego-right direction: front → left → back → right. Cam1 is positioned at the front (closest to the viewer), and Cam2 is positioned to the left of Cam1. Since the first image is at the beginning and the second image is at the end, the camera must have moved from front to left — which is a counter-clockwise (left) orbit.
+In the 3D view, Cam1 is positioned to the right of the object (green mug), and Cam2 is positioned to the left. The mug is centered in the scene. The camera movement from Cam1 to Cam2 is a leftward movement, meaning the camera is orbiting counter-clockwise — which corresponds to “left” in the problem’s directionality.
+We must verify this against the original images. In the first image (Cam1), the mug is centered and the camera is slightly to the right of the mug. In the second image (Cam2), the mug is still centered, but the camera has moved to the left. This confirms the leftward movement.
+Thus, the camera is moving left.
+&lt;answer&gt;(A) left&lt;/answer&gt;</t>
   </si>
   <si>
     <t>The two images show a static scene with a green mug centered on a checkered tablecloth. In the first image, the mug is centered, and the camera appears to be facing directly toward it. In the second image, the mug is still centered, but the perspective has shifted: the mug’s handle and the left side of the mug are now more prominent, and the background elements (coffee cans, flowers) appear to have moved slightly to the right relative to the mug’s position.
@@ -1955,11 +1955,11 @@
 &lt;answer&gt;B&lt;/answer&gt;</t>
   </si>
   <si>
-    <t>The unresolved geometric quantity is the lateral displacement sign of the person in relation to the bottle, as the initial conclusion based on relative positions may be ambiguous without a global reference.
-To resolve this, I will use the second method: request a second GLOBAL view with camera_view=false, rotation_reference_camera=1, and a substantially different nonzero angle. I will reproject C2-C1 into cam1's frame to verify the lateral sign.
-This will help confirm whether the person was on the left or right side of the bottle in the first frame relative to the camera’s orbit direction.
-After obtaining the second view, I will inspect the forward central ray and far scene boundary to verify the orbit direction.
-&lt;answer&gt;(A) left&lt;/answer&gt;</t>
+    <t>The unresolved geometric quantity is: **lateral displacement sign** — specifically, whether the camera moved left (clockwise) or right (counter-clockwise) around the object.
+To resolve this, we must compare the relative positions of the object (bottle) and background elements between the two images. In the first image, the person in the red shirt is visible to the left of the bottle. In the second image, the person is no longer visible, and the background has shifted to show shelves and a different part of the store. This suggests the camera has moved from a position where the person is on the left to a position where the person is no longer in the frame — consistent with a **clockwise (right)** rotation.
+Additionally, the second image shows the bottle’s position relative to the pink bag — in the first image, the bottle is to the left of the bag; in the second, the bottle is centered with the bag to its left. This lateral shift confirms the camera has rotated right.
+Thus, the camera is moving **right**.
+&lt;answer&gt;B&lt;/answer&gt;</t>
   </si>
 </sst>
 </file>

</xml_diff>